<commit_message>
last 2 lines of home loan
</commit_message>
<xml_diff>
--- a/testdata/EMIData.xlsx
+++ b/testdata/EMIData.xlsx
@@ -23,10 +23,10 @@
     <t>₹ 16,747</t>
   </si>
   <si>
-    <t>₹ 1,50,15,125</t>
-  </si>
-  <si>
-    <t>₹ 1,50,40,154</t>
+    <t>₹ 1,50,24,175</t>
+  </si>
+  <si>
+    <t>₹ 1,50,49,204</t>
   </si>
   <si>
     <t>₹ 4,41,717</t>
@@ -44,10 +44,10 @@
     <t>₹ 32,535</t>
   </si>
   <si>
-    <t>₹ 3,00,30,250</t>
-  </si>
-  <si>
-    <t>₹ 3,00,80,309</t>
+    <t>₹ 3,00,48,350</t>
+  </si>
+  <si>
+    <t>₹ 3,00,98,409</t>
   </si>
   <si>
     <t>₹ 4,24,193</t>

</xml_diff>